<commit_message>
chore: update coding-agents leaderboard (2026-08-21)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_coding_agents.xlsx
+++ b/data/artificial_analysis_coding_agents.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T47"/>
+  <dimension ref="A1:T56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3738,6 +3738,636 @@
         <v>8152.734606749675</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Cursor CLI</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Composer 2.5 Fast</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>cursor</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0.3830075380367747</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.15929203539823</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.6779026217228465</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.3118279569892475</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0.5573437730061347</v>
+      </c>
+      <c r="J48" t="n">
+        <v>472.3722024539875</v>
+      </c>
+      <c r="K48" t="n">
+        <v>116.8680981595092</v>
+      </c>
+      <c r="L48" t="n">
+        <v>4259887.413087938</v>
+      </c>
+      <c r="M48" t="n">
+        <v>2153033.982617587</v>
+      </c>
+      <c r="N48" t="n">
+        <v>20146.14621676892</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0.9355410155352529</v>
+      </c>
+      <c r="P48" t="n">
+        <v>0.6872016098268293</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>8.991024900330346e-05</v>
+      </c>
+      <c r="R48" t="n">
+        <v>0.04864903599920222</v>
+      </c>
+      <c r="S48" t="n">
+        <v>1.455177033493845</v>
+      </c>
+      <c r="T48" t="n">
+        <v>9018.073864121761</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Opus 5 (xhigh)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0.6814975428587521</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.6047197640118001</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.891385767790262</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.5483870967741939</v>
+      </c>
+      <c r="I49" t="n">
+        <v>8.170783921523503</v>
+      </c>
+      <c r="J49" t="n">
+        <v>1421.879982617586</v>
+      </c>
+      <c r="K49" t="n">
+        <v>152.0771983640082</v>
+      </c>
+      <c r="L49" t="n">
+        <v>21565879.13803684</v>
+      </c>
+      <c r="M49" t="n">
+        <v>10747525.6196319</v>
+      </c>
+      <c r="N49" t="n">
+        <v>73273.02862985685</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0.9740249879523308</v>
+      </c>
+      <c r="P49" t="n">
+        <v>0.08340662896047824</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>3.160073088125399e-05</v>
+      </c>
+      <c r="R49" t="n">
+        <v>0.0287575977377849</v>
+      </c>
+      <c r="S49" t="n">
+        <v>11.98945470477945</v>
+      </c>
+      <c r="T49" t="n">
+        <v>15167.15855183185</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Grok Build</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Grok 4.5 (high)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>xai</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>0.6408998279698193</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.59882005899705</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.842696629213483</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0.481182795698925</v>
+      </c>
+      <c r="I50" t="n">
+        <v>2.438982443762777</v>
+      </c>
+      <c r="J50" t="n">
+        <v>929.185109406954</v>
+      </c>
+      <c r="K50" t="n">
+        <v>60.74437627811862</v>
+      </c>
+      <c r="L50" t="n">
+        <v>3598867.582822087</v>
+      </c>
+      <c r="M50" t="n">
+        <v>1837535.160531697</v>
+      </c>
+      <c r="N50" t="n">
+        <v>25699.40797546012</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0.9238990226060745</v>
+      </c>
+      <c r="P50" t="n">
+        <v>0.2627734486604427</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>0.0001780837480736792</v>
+      </c>
+      <c r="R50" t="n">
+        <v>0.04138463831252327</v>
+      </c>
+      <c r="S50" t="n">
+        <v>3.805559523223389</v>
+      </c>
+      <c r="T50" t="n">
+        <v>3873.143840110653</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Kimi Code CLI</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>moonshotai</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>0.6263880112748017</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.63716814159292</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.8764044943820229</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0.365591397849462</v>
+      </c>
+      <c r="I51" t="n">
+        <v>3.081635541610432</v>
+      </c>
+      <c r="J51" t="n">
+        <v>1447.373053169734</v>
+      </c>
+      <c r="K51" t="n">
+        <v>122.9498977505112</v>
+      </c>
+      <c r="L51" t="n">
+        <v>10383196.73788345</v>
+      </c>
+      <c r="M51" t="n">
+        <v>5296768.575664621</v>
+      </c>
+      <c r="N51" t="n">
+        <v>54498.01533742331</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0.9500000000000018</v>
+      </c>
+      <c r="P51" t="n">
+        <v>0.2032647932621707</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>6.032708683920082e-05</v>
+      </c>
+      <c r="R51" t="n">
+        <v>0.02596654718296782</v>
+      </c>
+      <c r="S51" t="n">
+        <v>4.919691127770471</v>
+      </c>
+      <c r="T51" t="n">
+        <v>7173.822060003357</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Opencode</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Gemini 3.7 Flash (high)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>SST</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>0.5962784529614886</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.572271386430678</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.910112359550562</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.306451612903226</v>
+      </c>
+      <c r="I52" t="n">
+        <v>1.26793256886503</v>
+      </c>
+      <c r="J52" t="n">
+        <v>527.0915644171779</v>
+      </c>
+      <c r="K52" t="n">
+        <v>83.44887525562373</v>
+      </c>
+      <c r="L52" t="n">
+        <v>18493123.37423313</v>
+      </c>
+      <c r="M52" t="n">
+        <v>9497213.109406954</v>
+      </c>
+      <c r="N52" t="n">
+        <v>49098.7944785276</v>
+      </c>
+      <c r="O52" t="n">
+        <v>0.8634331167917663</v>
+      </c>
+      <c r="P52" t="n">
+        <v>0.4702761547447575</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>3.224325285107308e-05</v>
+      </c>
+      <c r="R52" t="n">
+        <v>0.06787569673449199</v>
+      </c>
+      <c r="S52" t="n">
+        <v>2.126410173917388</v>
+      </c>
+      <c r="T52" t="n">
+        <v>35085.21976571864</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Fable 5 (max) (with fallback)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0.6717276042685724</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.660766961651917</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.865168539325843</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0.489247311827957</v>
+      </c>
+      <c r="I53" t="n">
+        <v>11.68740762091003</v>
+      </c>
+      <c r="J53" t="n">
+        <v>1407.30630163599</v>
+      </c>
+      <c r="K53" t="n">
+        <v>137.007744236847</v>
+      </c>
+      <c r="L53" t="n">
+        <v>13868659.99897749</v>
+      </c>
+      <c r="M53" t="n">
+        <v>6901095.023517382</v>
+      </c>
+      <c r="N53" t="n">
+        <v>74265.48875255625</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0.9619283373252908</v>
+      </c>
+      <c r="P53" t="n">
+        <v>0.05747447390016408</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>4.843493202069251e-05</v>
+      </c>
+      <c r="R53" t="n">
+        <v>0.02863886576025522</v>
+      </c>
+      <c r="S53" t="n">
+        <v>17.39902833624972</v>
+      </c>
+      <c r="T53" t="n">
+        <v>9854.75584302807</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>GLM-5.2</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>novita</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0.4331015719360217</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.286135693215339</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.722846441947565</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0.290322580645161</v>
+      </c>
+      <c r="I54" t="n">
+        <v>6.657531358159519</v>
+      </c>
+      <c r="J54" t="n">
+        <v>1507.044470347651</v>
+      </c>
+      <c r="K54" t="n">
+        <v>127.4036879531512</v>
+      </c>
+      <c r="L54" t="n">
+        <v>6619529.539877302</v>
+      </c>
+      <c r="M54" t="n">
+        <v>5529735.922290388</v>
+      </c>
+      <c r="N54" t="n">
+        <v>28567.83231083845</v>
+      </c>
+      <c r="O54" t="n">
+        <v>0.3295602231414034</v>
+      </c>
+      <c r="P54" t="n">
+        <v>0.06505437956446262</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>6.542784790473939e-05</v>
+      </c>
+      <c r="R54" t="n">
+        <v>0.01724308394838987</v>
+      </c>
+      <c r="S54" t="n">
+        <v>15.37175524069208</v>
+      </c>
+      <c r="T54" t="n">
+        <v>4392.391644786887</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Flash (max)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>0.497576003161905</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.427728613569321</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.677902621722846</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.387096774193548</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0.05949917044417183</v>
+      </c>
+      <c r="J55" t="n">
+        <v>868.3750143149272</v>
+      </c>
+      <c r="K55" t="n">
+        <v>105.9314928425358</v>
+      </c>
+      <c r="L55" t="n">
+        <v>20844227.99386501</v>
+      </c>
+      <c r="M55" t="n">
+        <v>10443571.69734151</v>
+      </c>
+      <c r="N55" t="n">
+        <v>58411.25766871166</v>
+      </c>
+      <c r="O55" t="n">
+        <v>0.9807621661364226</v>
+      </c>
+      <c r="P55" t="n">
+        <v>8.362738496140571</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>2.38711648763559e-05</v>
+      </c>
+      <c r="R55" t="n">
+        <v>0.03437980100483081</v>
+      </c>
+      <c r="S55" t="n">
+        <v>0.1195780545405674</v>
+      </c>
+      <c r="T55" t="n">
+        <v>24003.71688527831</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Sol (max)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>0.6505240024334411</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.687315634218289</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0.831460674157303</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0.432795698924731</v>
+      </c>
+      <c r="I56" t="n">
+        <v>6.420249160020451</v>
+      </c>
+      <c r="J56" t="n">
+        <v>613.70177198364</v>
+      </c>
+      <c r="K56" t="n">
+        <v>112.2689161554192</v>
+      </c>
+      <c r="L56" t="n">
+        <v>13169248.79601226</v>
+      </c>
+      <c r="M56" t="n">
+        <v>6786107.398261759</v>
+      </c>
+      <c r="N56" t="n">
+        <v>35184.01329243354</v>
+      </c>
+      <c r="O56" t="n">
+        <v>0.902597320865973</v>
+      </c>
+      <c r="P56" t="n">
+        <v>0.1013237938621324</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>4.939719892226686e-05</v>
+      </c>
+      <c r="R56" t="n">
+        <v>0.06360001213593849</v>
+      </c>
+      <c r="S56" t="n">
+        <v>9.869350148501775</v>
+      </c>
+      <c r="T56" t="n">
+        <v>21458.71072434076</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>